<commit_message>
Update process document templates
</commit_message>
<xml_diff>
--- a/public/templates/process-docs/UPS装置检查及带负荷试验分项工程质量检查验收评定表.xlsx
+++ b/public/templates/process-docs/UPS装置检查及带负荷试验分项工程质量检查验收评定表.xlsx
@@ -57,7 +57,7 @@
     <t xml:space="preserve">工程编号：</t>
   </si>
   <si>
-    <t xml:space="preserve">5028G01-0011</t>
+    <t xml:space="preserve">{{工程编号}}</t>
   </si>
   <si>
     <t xml:space="preserve">性质：</t>
@@ -112,37 +112,37 @@
     <t xml:space="preserve">总承包单位</t>
   </si>
   <si>
-    <t xml:space="preserve">中核华辰建筑工程有限公司</t>
+    <t xml:space="preserve">{{施工单位}}</t>
   </si>
   <si>
     <t xml:space="preserve">项目负责人</t>
   </si>
   <si>
-    <t xml:space="preserve">谢智敏</t>
+    <t xml:space="preserve">{{施工单位项目负责人}}</t>
   </si>
   <si>
     <t xml:space="preserve">项目技术负责人</t>
   </si>
   <si>
-    <t xml:space="preserve">蒋志炜</t>
+    <t xml:space="preserve">{{总承包单位项目技术负责人}}</t>
   </si>
   <si>
     <t xml:space="preserve">施工单位</t>
   </si>
   <si>
-    <t xml:space="preserve">刘彦堂</t>
+    <t xml:space="preserve">{{施工单位项目技术负责人}}</t>
   </si>
   <si>
     <t xml:space="preserve">分包单位</t>
   </si>
   <si>
-    <t xml:space="preserve">河南誉华美建设工程有限公司</t>
+    <t xml:space="preserve">{{分包单位}}</t>
   </si>
   <si>
     <t xml:space="preserve">分包项目负责人</t>
   </si>
   <si>
-    <t xml:space="preserve">胡彦芳</t>
+    <t xml:space="preserve">{{分包单位项目负责人}}</t>
   </si>
   <si>
     <t xml:space="preserve">分包内容</t>

</xml_diff>